<commit_message>
Translated dataset and updated Albanian files
</commit_message>
<xml_diff>
--- a/datasets/MECO-dataset/release 1.0/auxiliary files/reading task materials/supp texts.xlsx
+++ b/datasets/MECO-dataset/release 1.0/auxiliary files/reading task materials/supp texts.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB5E434-1615-4628-9DDC-26804C5E4ADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{784B092C-8500-4D21-92F1-98B7F22AF09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -571,7 +571,7 @@
     <t>Albanian</t>
   </si>
   <si>
-    <t>Në fenë dhe mitin e lashtë romak, Janusi është perëndia e fillimeve dhe portave. Ai ka një natyrë të dyfishtë dhe zakonisht përshkruhet si me dy fytyra, pasi shikon drejt së ardhmes dhe të kaluarës. Janusi kryesonte fillimin dhe mbarimin e konfliktit, dhe për rrjedhojë luftën dhe paqen. Dyert e tempullit të tij ishin të hapura në kohë lufte dhe të mbyllura gjatë kohës së paqes. Si perëndia e portave, ai shoqërohej gjithashtu me hyrjen dhe daljen nga dyert e shtëpive. Janusi shpesh simbolizonte ndryshimin dhe tranzicionet, të tilla si përparimi nga një gjendje në tjetrën, nga një vizion në tjetrin dhe rritja e të rinjve në moshë madhore. Prandaj, Janusi adhurohej në fillim të kohës së korrjes dhe mbjelljes, si dhe në martesa, vdekje dhe fillime të tjera. Janusi nuk kishte një prift të specializuar të caktuar për të, por vetë kryeprifti kryente ceremonitë e tij. Janusi përfaqësonte terrenin e mesëm midis barbarizmit dhe qytetërimit, hapësirës rurale dhe urbane, rinisë dhe moshës madhore. Grekët e lashtë nuk kishin ekuivalent me Janusin, të cilin romakët e pretendonin si të tyren.</t>
+    <t>Në fenë dhe mitin e lashtë romak, Janusi është perëndia e fillimeve dhe portave. Ai ka një natyrë të dyfishtë dhe zakonisht përshkruhet si me dy fytyra, pasi shikon drejt së ardhmes dhe të kaluarës. Janusi kryesonte fillimin dhe mbarimin e konfliktit, dhe për rrjedhojë luftën dhe paqen. Dyert e tempullit të tij ishin të hapura në kohë lufte dhe të mbyllura gjatë kohës së paqes. Si zot i portave, ai shoqërohej edhe me aktin e hyrjes dhe daljes nga dyert e shtëpive. Janusi shpesh simbolizonte ndryshimin dhe tranzicionet, të tilla si përparimi nga një gjendje në tjetrën, nga një vizion në tjetrin dhe rritja e të rinjve në moshë madhore. Prandaj, Janusi adhurohej në fillim të kohës së korrjes dhe mbjelljes, si dhe në martesa, vdekje dhe fillime të tjera. Janusi nuk kishte një prift të specializuar të caktuar për të, por vetë kryeprifti kryente ceremonitë e tij. Janusi përfaqësonte terrenin e mesëm midis barbarizmit dhe qytetërimit, hapësirës rurale dhe urbane, rinisë dhe moshës madhore. Grekët e lashtë nuk kishin ekuivalent me Janusin, të cilin romakët e pretendonin si të tyren.</t>
   </si>
 </sst>
 </file>
@@ -627,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -642,6 +642,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -923,14 +926,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O25"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.6328125" style="1"/>
-    <col min="2" max="13" width="255.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.6328125" style="1"/>
+    <col min="1" max="1" width="8.6640625" style="1"/>
+    <col min="2" max="13" width="255.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="2" t="s">
         <v>12</v>
       </c>
@@ -969,7 +972,7 @@
       </c>
       <c r="O1" s="3"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1011,7 +1014,7 @@
       </c>
       <c r="O2" s="3"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -1053,7 +1056,7 @@
       </c>
       <c r="O3" s="3"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>168</v>
       </c>
@@ -1095,7 +1098,7 @@
       </c>
       <c r="O4" s="3"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
@@ -1137,7 +1140,7 @@
       </c>
       <c r="O5" s="3"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
@@ -1179,7 +1182,7 @@
       </c>
       <c r="O6" s="3"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -1221,7 +1224,7 @@
       </c>
       <c r="O7" s="3"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>5</v>
       </c>
@@ -1263,7 +1266,7 @@
       </c>
       <c r="O8" s="3"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>6</v>
       </c>
@@ -1305,7 +1308,7 @@
       </c>
       <c r="O9" s="3"/>
     </row>
-    <row r="10" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
@@ -1347,7 +1350,7 @@
       </c>
       <c r="O10" s="3"/>
     </row>
-    <row r="11" spans="1:15" ht="26" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
@@ -1389,7 +1392,7 @@
       </c>
       <c r="O11" s="3"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
@@ -1431,7 +1434,7 @@
       </c>
       <c r="O12" s="3"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>10</v>
       </c>
@@ -1473,7 +1476,7 @@
       </c>
       <c r="O13" s="3"/>
     </row>
-    <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>11</v>
       </c>
@@ -1515,43 +1518,43 @@
       </c>
       <c r="O14" s="3"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="6" t="s">
         <v>182</v>
       </c>
       <c r="O15" s="3"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="O16" s="3"/>
     </row>
-    <row r="17" spans="15:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="15:15" x14ac:dyDescent="0.3">
       <c r="O17" s="3"/>
     </row>
-    <row r="18" spans="15:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="15:15" x14ac:dyDescent="0.3">
       <c r="O18" s="3"/>
     </row>
-    <row r="19" spans="15:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="15:15" x14ac:dyDescent="0.3">
       <c r="O19" s="3"/>
     </row>
-    <row r="20" spans="15:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="15:15" x14ac:dyDescent="0.3">
       <c r="O20" s="3"/>
     </row>
-    <row r="21" spans="15:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="15:15" x14ac:dyDescent="0.3">
       <c r="O21" s="3"/>
     </row>
-    <row r="22" spans="15:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="15:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="O22" s="3"/>
     </row>
-    <row r="23" spans="15:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="15:15" x14ac:dyDescent="0.3">
       <c r="O23" s="3"/>
     </row>
-    <row r="24" spans="15:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="15:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="O24" s="3"/>
     </row>
-    <row r="25" spans="15:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="15:15" x14ac:dyDescent="0.3">
       <c r="O25" s="3"/>
     </row>
   </sheetData>

</xml_diff>